<commit_message>
agregacion de nueva tabla
</commit_message>
<xml_diff>
--- a/uploads/ZSD058_260407_5PM_III.XLSX
+++ b/uploads/ZSD058_260407_5PM_III.XLSX
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\17. Programación de Producción\07. PROYECTO SOFTWARE PROG PROD\2025 IT\Entregable 260407\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\atecnologia2\Documents\PROYECTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7530"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21600" windowHeight="9630"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -917,7 +917,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T61"/>
+  <dimension ref="A1:R61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -938,7 +938,7 @@
     <col min="18" max="18" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>166</v>
       </c>
@@ -993,11 +993,8 @@
       <c r="R1" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="T1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>20347404</v>
       </c>
@@ -1053,7 +1050,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>20347405</v>
       </c>
@@ -1109,7 +1106,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>20347406</v>
       </c>
@@ -1165,7 +1162,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>20347407</v>
       </c>
@@ -1221,7 +1218,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>20347408</v>
       </c>
@@ -1277,7 +1274,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>20347701</v>
       </c>
@@ -1333,7 +1330,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>20347702</v>
       </c>
@@ -1389,7 +1386,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>20347703</v>
       </c>
@@ -1445,7 +1442,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>20347704</v>
       </c>
@@ -1501,7 +1498,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>20347705</v>
       </c>
@@ -1557,7 +1554,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>20347706</v>
       </c>
@@ -1613,7 +1610,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>20347707</v>
       </c>
@@ -1669,7 +1666,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>20347708</v>
       </c>
@@ -1725,7 +1722,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>20347709</v>
       </c>
@@ -1781,7 +1778,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>20347710</v>
       </c>

</xml_diff>